<commit_message>
This commit for final project
</commit_message>
<xml_diff>
--- a/src/test/resources/Data/UserTestData.xlsx
+++ b/src/test/resources/Data/UserTestData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmurugan\eclipse-workspace\FinalProject\src\test\resources\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A324A3D6-BC98-4D21-910F-16AFDF15FC9D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F9AE74C-8396-4913-A1E4-854235DBBF26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="5" activeTab="9" xr2:uid="{71A006D7-44F9-41BE-B93B-F960204E6E39}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" firstSheet="4" activeTab="4" xr2:uid="{71A006D7-44F9-41BE-B93B-F960204E6E39}"/>
   </bookViews>
   <sheets>
     <sheet name="Login" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1481" uniqueCount="202">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1538" uniqueCount="203">
   <si>
     <t>Username</t>
   </si>
@@ -652,6 +652,9 @@
   </si>
   <si>
     <t>username</t>
+  </si>
+  <si>
+    <t>ram1278923@gmail.com</t>
   </si>
 </sst>
 </file>
@@ -1528,7 +1531,7 @@
         <v>186</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>187</v>
+        <v>202</v>
       </c>
       <c r="F15" s="1" t="s">
         <v>13</v>
@@ -5244,7 +5247,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DC6ABA4-852F-4513-943D-173D31D839A7}">
-  <dimension ref="A1:T10"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.77734375" bestFit="1" customWidth="1"/>
@@ -5858,6 +5861,183 @@
         <v>13</v>
       </c>
     </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="M11" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="N11" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="S11" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="N12" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="O12" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="P12" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="S12" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="N13" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="S13" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>